<commit_message>
Fix Salesinvoice Product Details margin and percentage columns
The Product Details sheet's Gross Profit Margin column (G) carried the
percentage formula instead of the margin, and the Gross Profit Margin %
column (H) was empty, for every product row. Column G now computes
C-F and column H carries the percentage, using new shared formula
groups (si=2 for rows 6-66, si=3 for rows 67-99) so the guard can see
the H column is covered.

The template also ships a second shared group at G67:G99 (si=1) with
the identical defect, one row block below the G6:G66 group the repair
plan described. Fixed both groups; the plan's write-up only covered
the first.

Verified with a full unzipped directory diff against the pre-repair
template: only xl/worksheets/sheet4.xml changed in each workbook.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Salesinvoice.xlsx
+++ b/app/templates/ltd/Salesinvoice.xlsx
@@ -7801,10 +7801,13 @@
         <v>20</v>
       </c>
       <c r="G6" s="63" t="str">
-        <f t="shared" ref="G6:G66" si="0">IF(F6&gt;0,(C6-F6)*100/C6," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H6" s="64"/>
+        <f t="shared" ref="G6:G66" si="0">IF(F6&gt;0,C6-F6," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H6" s="64" t="str">
+        <f t="shared" ref="H6:H66" si="2">IF(F6&gt;0,(C6-F6)*100/C6," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D7" s="56">
@@ -7814,7 +7817,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H7" s="64"/>
+      <c r="H7" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D8" s="56">
@@ -7824,7 +7830,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H8" s="64"/>
+      <c r="H8" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D9" s="56">
@@ -7834,7 +7843,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H9" s="64"/>
+      <c r="H9" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D10" s="56">
@@ -7844,7 +7856,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H10" s="64"/>
+      <c r="H10" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D11" s="56">
@@ -7854,7 +7869,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H11" s="64"/>
+      <c r="H11" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D12" s="56">
@@ -7864,7 +7882,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H12" s="64"/>
+      <c r="H12" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D13" s="56">
@@ -7874,7 +7895,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H13" s="64"/>
+      <c r="H13" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D14" s="56">
@@ -7884,7 +7908,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H14" s="64"/>
+      <c r="H14" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D15" s="56">
@@ -7894,7 +7921,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H15" s="64"/>
+      <c r="H15" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D16" s="56">
@@ -7904,7 +7934,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H16" s="64"/>
+      <c r="H16" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="17" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D17" s="56">
@@ -7914,7 +7947,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H17" s="64"/>
+      <c r="H17" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="18" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D18" s="56">
@@ -7924,7 +7960,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H18" s="64"/>
+      <c r="H18" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="19" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D19" s="56">
@@ -7934,7 +7973,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H19" s="64"/>
+      <c r="H19" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D20" s="56">
@@ -7944,7 +7986,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H20" s="64"/>
+      <c r="H20" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="21" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D21" s="56">
@@ -7954,7 +7999,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H21" s="64"/>
+      <c r="H21" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="22" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D22" s="56">
@@ -7964,7 +8012,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H22" s="64"/>
+      <c r="H22" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="23" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D23" s="56">
@@ -7974,7 +8025,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H23" s="64"/>
+      <c r="H23" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="24" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D24" s="56">
@@ -7984,7 +8038,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H24" s="64"/>
+      <c r="H24" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="25" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D25" s="56">
@@ -7994,7 +8051,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H25" s="64"/>
+      <c r="H25" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="26" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D26" s="56">
@@ -8004,7 +8064,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H26" s="64"/>
+      <c r="H26" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="27" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D27" s="56">
@@ -8014,7 +8077,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H27" s="64"/>
+      <c r="H27" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="28" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D28" s="56">
@@ -8024,7 +8090,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H28" s="64"/>
+      <c r="H28" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="29" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D29" s="56">
@@ -8034,7 +8103,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H29" s="64"/>
+      <c r="H29" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="30" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D30" s="56">
@@ -8044,7 +8116,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H30" s="64"/>
+      <c r="H30" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="31" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D31" s="56">
@@ -8054,7 +8129,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H31" s="64"/>
+      <c r="H31" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="32" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D32" s="56">
@@ -8064,7 +8142,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H32" s="64"/>
+      <c r="H32" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="33" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D33" s="56">
@@ -8074,7 +8155,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H33" s="64"/>
+      <c r="H33" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="34" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D34" s="56">
@@ -8084,7 +8168,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H34" s="64"/>
+      <c r="H34" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="35" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D35" s="56">
@@ -8094,7 +8181,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H35" s="64"/>
+      <c r="H35" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="36" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D36" s="56">
@@ -8104,7 +8194,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H36" s="64"/>
+      <c r="H36" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="37" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D37" s="56">
@@ -8114,7 +8207,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H37" s="64"/>
+      <c r="H37" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="38" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D38" s="56">
@@ -8124,7 +8220,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H38" s="64"/>
+      <c r="H38" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="39" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D39" s="56">
@@ -8134,7 +8233,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H39" s="64"/>
+      <c r="H39" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="40" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D40" s="56">
@@ -8144,7 +8246,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H40" s="64"/>
+      <c r="H40" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="41" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D41" s="56">
@@ -8154,7 +8259,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H41" s="64"/>
+      <c r="H41" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="42" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D42" s="56">
@@ -8164,7 +8272,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H42" s="64"/>
+      <c r="H42" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="43" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D43" s="56">
@@ -8174,7 +8285,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H43" s="64"/>
+      <c r="H43" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="44" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D44" s="56">
@@ -8184,7 +8298,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H44" s="64"/>
+      <c r="H44" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="45" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D45" s="56">
@@ -8194,7 +8311,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H45" s="64"/>
+      <c r="H45" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="46" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D46" s="56">
@@ -8204,7 +8324,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H46" s="64"/>
+      <c r="H46" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="47" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D47" s="56">
@@ -8214,7 +8337,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H47" s="64"/>
+      <c r="H47" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="48" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D48" s="56">
@@ -8224,7 +8350,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H48" s="64"/>
+      <c r="H48" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="49" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D49" s="56">
@@ -8234,7 +8363,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H49" s="64"/>
+      <c r="H49" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="50" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D50" s="56">
@@ -8244,7 +8376,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H50" s="64"/>
+      <c r="H50" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="51" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D51" s="56">
@@ -8254,7 +8389,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H51" s="64"/>
+      <c r="H51" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="52" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D52" s="56">
@@ -8264,7 +8402,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H52" s="64"/>
+      <c r="H52" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="53" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D53" s="56">
@@ -8274,7 +8415,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H53" s="64"/>
+      <c r="H53" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="54" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D54" s="56">
@@ -8284,7 +8428,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H54" s="64"/>
+      <c r="H54" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="55" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D55" s="56">
@@ -8294,7 +8441,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H55" s="64"/>
+      <c r="H55" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="56" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D56" s="56">
@@ -8304,7 +8454,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H56" s="64"/>
+      <c r="H56" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="57" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D57" s="56">
@@ -8314,7 +8467,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H57" s="64"/>
+      <c r="H57" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="58" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D58" s="56">
@@ -8324,7 +8480,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H58" s="64"/>
+      <c r="H58" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="59" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D59" s="56">
@@ -8334,7 +8493,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H59" s="64"/>
+      <c r="H59" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="60" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D60" s="56">
@@ -8344,7 +8506,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H60" s="64"/>
+      <c r="H60" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="61" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D61" s="56">
@@ -8354,7 +8519,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H61" s="64"/>
+      <c r="H61" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="62" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D62" s="56">
@@ -8364,7 +8532,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H62" s="64"/>
+      <c r="H62" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="63" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D63" s="56">
@@ -8374,7 +8545,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H63" s="64"/>
+      <c r="H63" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="64" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D64" s="56">
@@ -8384,7 +8558,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H64" s="64"/>
+      <c r="H64" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="65" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D65" s="56">
@@ -8394,7 +8571,10 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H65" s="64"/>
+      <c r="H65" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="66" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D66" s="56">
@@ -8404,17 +8584,23 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H66" s="64"/>
+      <c r="H66" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="67" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D67" s="56">
         <v>20</v>
       </c>
       <c r="G67" s="63" t="str">
-        <f t="shared" ref="G67:G99" si="1">IF(F67&gt;0,(C67-F67)*100/C67," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H67" s="64"/>
+        <f t="shared" ref="G67:G99" si="1">IF(F67&gt;0,C67-F67," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H67" s="64" t="str">
+        <f t="shared" ref="H67:H99" si="3">IF(F67&gt;0,(C67-F67)*100/C67," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="68" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D68" s="56">
@@ -8424,7 +8610,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H68" s="64"/>
+      <c r="H68" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="69" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D69" s="56">
@@ -8434,7 +8623,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H69" s="64"/>
+      <c r="H69" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="70" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D70" s="56">
@@ -8444,7 +8636,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H70" s="64"/>
+      <c r="H70" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="71" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D71" s="56">
@@ -8454,7 +8649,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H71" s="64"/>
+      <c r="H71" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="72" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D72" s="56">
@@ -8464,7 +8662,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H72" s="64"/>
+      <c r="H72" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="73" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D73" s="56">
@@ -8474,7 +8675,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H73" s="64"/>
+      <c r="H73" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="74" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D74" s="56">
@@ -8484,7 +8688,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H74" s="64"/>
+      <c r="H74" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="75" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D75" s="56">
@@ -8494,7 +8701,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H75" s="64"/>
+      <c r="H75" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="76" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D76" s="56">
@@ -8504,7 +8714,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H76" s="64"/>
+      <c r="H76" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="77" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D77" s="56">
@@ -8514,7 +8727,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H77" s="64"/>
+      <c r="H77" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="78" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D78" s="56">
@@ -8524,7 +8740,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H78" s="64"/>
+      <c r="H78" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="79" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D79" s="56">
@@ -8534,7 +8753,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H79" s="64"/>
+      <c r="H79" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="80" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D80" s="56">
@@ -8544,7 +8766,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H80" s="64"/>
+      <c r="H80" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="81" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D81" s="56">
@@ -8554,7 +8779,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H81" s="64"/>
+      <c r="H81" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="82" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D82" s="56">
@@ -8564,7 +8792,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H82" s="64"/>
+      <c r="H82" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="83" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D83" s="56">
@@ -8574,7 +8805,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H83" s="64"/>
+      <c r="H83" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="84" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D84" s="56">
@@ -8584,7 +8818,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H84" s="64"/>
+      <c r="H84" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="85" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D85" s="56">
@@ -8594,7 +8831,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H85" s="64"/>
+      <c r="H85" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="86" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D86" s="56">
@@ -8604,7 +8844,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H86" s="64"/>
+      <c r="H86" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="87" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D87" s="56">
@@ -8614,7 +8857,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H87" s="64"/>
+      <c r="H87" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="88" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D88" s="56">
@@ -8624,7 +8870,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H88" s="64"/>
+      <c r="H88" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="89" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D89" s="56">
@@ -8634,7 +8883,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H89" s="64"/>
+      <c r="H89" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="90" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D90" s="56">
@@ -8644,7 +8896,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H90" s="64"/>
+      <c r="H90" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="91" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D91" s="56">
@@ -8654,7 +8909,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H91" s="64"/>
+      <c r="H91" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="92" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D92" s="56">
@@ -8664,7 +8922,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H92" s="64"/>
+      <c r="H92" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="93" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D93" s="56">
@@ -8674,7 +8935,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H93" s="64"/>
+      <c r="H93" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="94" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D94" s="56">
@@ -8684,7 +8948,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H94" s="64"/>
+      <c r="H94" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="95" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D95" s="56">
@@ -8694,7 +8961,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H95" s="64"/>
+      <c r="H95" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="96" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D96" s="56">
@@ -8704,7 +8974,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H96" s="64"/>
+      <c r="H96" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D97" s="56">
@@ -8714,7 +8987,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H97" s="64"/>
+      <c r="H97" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D98" s="56">
@@ -8724,7 +9000,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H98" s="64"/>
+      <c r="H98" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
     <row r="99" spans="1:8" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A99" s="57"/>
@@ -8738,7 +9017,10 @@
         <f t="shared" si="1"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H99" s="66"/>
+      <c r="H99" s="66" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>